<commit_message>
feat(import): support full entity fields and update test data
</commit_message>
<xml_diff>
--- a/test-data/clients.xlsx
+++ b/test-data/clients.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:L5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,27 @@
       <c r="E1" t="str">
         <v>Categoría</v>
       </c>
+      <c r="F1" t="str">
+        <v>Dirección</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Localidad</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Departamento</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Provincia</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Código Postal</v>
+      </c>
+      <c r="K1" t="str">
+        <v>País</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Teléfono</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,6 +453,27 @@
       <c r="E2" t="str">
         <v>cliente</v>
       </c>
+      <c r="F2" t="str">
+        <v>Av. 9 de Julio 1234</v>
+      </c>
+      <c r="G2" t="str">
+        <v>CABA</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Comuna 1</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Capital Federal</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1001</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="L2" t="str">
+        <v>11 4455-6677</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -449,6 +491,27 @@
       <c r="E3" t="str">
         <v>cliente</v>
       </c>
+      <c r="F3" t="str">
+        <v>Calle Falsa 123</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Rosario</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Rosario</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Santa Fe</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2000</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="L3" t="str">
+        <v>341 455-6677</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -466,6 +529,27 @@
       <c r="E4" t="str">
         <v>ambos</v>
       </c>
+      <c r="F4" t="str">
+        <v>Av. del Libertador 500</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Vicente López</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Vicente López</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Buenos Aires</v>
+      </c>
+      <c r="J4" t="str">
+        <v>1638</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="L4" t="str">
+        <v>11 3322-1100</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -483,10 +567,31 @@
       <c r="E5" t="str">
         <v>cliente</v>
       </c>
+      <c r="F5" t="str">
+        <v>Ruta 20 km 5</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Córdoba</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Capital</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Córdoba</v>
+      </c>
+      <c r="J5" t="str">
+        <v>5000</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="L5" t="str">
+        <v>351 998-8776</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>